<commit_message>
Updated plots and scripts
</commit_message>
<xml_diff>
--- a/output/tables/QC/finished_tables/Linkage_Disequilibrium.xlsx
+++ b/output/tables/QC/finished_tables/Linkage_Disequilibrium.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\R_WD\revised_bison_popgen\output\tables\QC\finished_tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D_RWD\revised_bison_popgen\output\tables\QC\finished_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9BE623A-02D4-4B07-9A36-956FA5CF8F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7250A611-9848-4869-8F9F-3C3CB56532CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-118" yWindow="-118" windowWidth="20343" windowHeight="12934" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="37">
   <si>
     <t>EINPW</t>
   </si>
@@ -147,12 +147,33 @@
   <si>
     <t>&lt;0.001</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Chromosomal Location</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,6 +210,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -266,25 +294,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,55 +596,55 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1"/>
-    <col min="4" max="4" width="4.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="4.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1"/>
+    <col min="4" max="4" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85546875" style="1"/>
+    <col min="6" max="6" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="1"/>
+    <col min="9" max="9" width="15.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="17.05" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="17.100000000000001" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" s="14" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -648,37 +676,37 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="10"/>
-      <c r="B3" s="12" t="s">
+      <c r="A3" s="15"/>
+      <c r="B3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="11">
         <v>8</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="11">
         <v>22</v>
       </c>
-      <c r="G3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" s="13">
+      <c r="G3" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="11">
         <v>41971</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="12" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="11"/>
+      <c r="A4" s="16"/>
       <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
@@ -708,39 +736,39 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="11">
         <v>1</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="11">
         <v>10</v>
       </c>
-      <c r="G5" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I5" s="13">
+      <c r="G5" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="11">
         <v>62199</v>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="11">
         <v>4.8216000000000002E-2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
+      <c r="A6" s="15"/>
       <c r="B6" s="4" t="s">
         <v>9</v>
       </c>
@@ -770,37 +798,37 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="10"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="15"/>
+      <c r="B7" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="11">
         <v>27</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="11">
         <v>7</v>
       </c>
-      <c r="G7" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="13">
+      <c r="G7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="11">
         <v>24169</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="12" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="10"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
@@ -830,37 +858,37 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="15"/>
+      <c r="B9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="11">
         <v>13</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="11">
         <v>5</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" s="13">
+      <c r="G9" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="11">
         <v>27811</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="12" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
+      <c r="A10" s="15"/>
       <c r="B10" s="4" t="s">
         <v>21</v>
       </c>
@@ -890,37 +918,37 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="15"/>
+      <c r="B11" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="11">
         <v>12</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="11">
         <v>15</v>
       </c>
-      <c r="G11" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" s="13">
+      <c r="G11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I11" s="11">
         <v>25452</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="11">
         <v>1.5679999999999999E-2</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="5" t="s">
         <v>21</v>
       </c>
@@ -949,7 +977,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="14.45" x14ac:dyDescent="0.25">
       <c r="E15" s="8"/>
     </row>
   </sheetData>

</xml_diff>